<commit_message>
Standardize analytics metrics and project documentation
</commit_message>
<xml_diff>
--- a/supply-chain-performance-analysis/excel_analysis/Supplychain_Dashboard.xlsx
+++ b/supply-chain-performance-analysis/excel_analysis/Supplychain_Dashboard.xlsx
@@ -820,17 +820,17 @@
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>$82.7M</t>
+          <t>$73.0M</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>$30.9M</t>
+          <t>$21.2M</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>37.4%</t>
+          <t>28.4%</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -886,7 +886,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>14.81</v>
+        <v>13.15</v>
       </c>
     </row>
     <row r="3">
@@ -896,7 +896,7 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>34.04</v>
+        <v>30.06</v>
       </c>
     </row>
     <row r="4">
@@ -906,7 +906,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>24.63</v>
+        <v>21.67</v>
       </c>
     </row>
     <row r="5">
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>9.210000000000001</v>
+        <v>8.16</v>
       </c>
     </row>
     <row r="7">
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="17">
@@ -1020,7 +1020,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>2.45</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="18">
@@ -1030,7 +1030,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>2.71</v>
+        <v>2.39</v>
       </c>
     </row>
     <row r="19">
@@ -1040,7 +1040,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>2.91</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="20">
@@ -1050,7 +1050,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>2.8</v>
+        <v>2.45</v>
       </c>
     </row>
     <row r="21">
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>2.32</v>
+        <v>2.06</v>
       </c>
     </row>
     <row r="22">
@@ -1070,7 +1070,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>2.98</v>
+        <v>2.66</v>
       </c>
     </row>
     <row r="23">
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="B23" s="5" t="n">
-        <v>3.05</v>
+        <v>2.71</v>
       </c>
     </row>
     <row r="24">
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>3.08</v>
+        <v>2.71</v>
       </c>
     </row>
     <row r="25">
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="B25" s="5" t="n">
-        <v>2.17</v>
+        <v>1.94</v>
       </c>
     </row>
     <row r="26">
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>2.2</v>
+        <v>1.93</v>
       </c>
     </row>
     <row r="27">
@@ -1120,7 +1120,7 @@
         </is>
       </c>
       <c r="B27" s="5" t="n">
-        <v>2.84</v>
+        <v>2.49</v>
       </c>
     </row>
     <row r="28">
@@ -1130,7 +1130,7 @@
         </is>
       </c>
       <c r="B28" s="5" t="n">
-        <v>2.8</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="29">
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="B29" s="5" t="n">
-        <v>2.6</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="30">
@@ -1150,7 +1150,7 @@
         </is>
       </c>
       <c r="B30" s="5" t="n">
-        <v>2.3</v>
+        <v>2.01</v>
       </c>
     </row>
     <row r="31">
@@ -1160,7 +1160,7 @@
         </is>
       </c>
       <c r="B31" s="5" t="n">
-        <v>2.65</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="32">
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="B32" s="5" t="n">
-        <v>2.61</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="33">
@@ -1180,7 +1180,7 @@
         </is>
       </c>
       <c r="B33" s="5" t="n">
-        <v>2.5</v>
+        <v>2.18</v>
       </c>
     </row>
     <row r="34">
@@ -1190,7 +1190,7 @@
         </is>
       </c>
       <c r="B34" s="5" t="n">
-        <v>3.07</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="35">
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>2.73</v>
+        <v>2.41</v>
       </c>
     </row>
     <row r="36">
@@ -1210,7 +1210,7 @@
         </is>
       </c>
       <c r="B36" s="5" t="n">
-        <v>3.13</v>
+        <v>2.81</v>
       </c>
     </row>
     <row r="37">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="B37" s="5" t="n">
-        <v>2.76</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="38">
@@ -1230,7 +1230,7 @@
         </is>
       </c>
       <c r="B38" s="5" t="n">
-        <v>2.31</v>
+        <v>2.05</v>
       </c>
     </row>
     <row r="39">
@@ -1240,7 +1240,7 @@
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>2.49</v>
+        <v>2.21</v>
       </c>
     </row>
     <row r="40">
@@ -1250,7 +1250,7 @@
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>2.78</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="41">
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>2.35</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="42">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="B42" s="5" t="n">
-        <v>3.11</v>
+        <v>2.77</v>
       </c>
     </row>
     <row r="43">
@@ -1280,7 +1280,7 @@
         </is>
       </c>
       <c r="B43" s="5" t="n">
-        <v>2.49</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="44">
@@ -1290,7 +1290,7 @@
         </is>
       </c>
       <c r="B44" s="5" t="n">
-        <v>2.38</v>
+        <v>2.09</v>
       </c>
     </row>
     <row r="45">
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="B45" s="5" t="n">
-        <v>2.78</v>
+        <v>2.42</v>
       </c>
     </row>
     <row r="46">
@@ -1310,7 +1310,7 @@
         </is>
       </c>
       <c r="B46" s="5" t="n">
-        <v>2.63</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="47">
@@ -1320,7 +1320,7 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>2.65</v>
+        <v>2.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>